<commit_message>
fix: mapas de carrera sin comisiones duplicadas, iconos refinados, cohesion de colores y terminos legales formalizados
</commit_message>
<xml_diff>
--- a/data/mapas/Mapa_de_Carrera_Psicologia.xlsx
+++ b/data/mapas/Mapa_de_Carrera_Psicologia.xlsx
@@ -62,14 +62,14 @@
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="0064748B"/>
-      <sz val="9"/>
+      <b val="1"/>
+      <color rgb="000B2545"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="000B2545"/>
-      <sz val="11"/>
+      <i val="1"/>
+      <sz val="8.5"/>
     </font>
   </fonts>
   <fills count="9">
@@ -87,26 +87,26 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="000284C7"/>
+        <bgColor rgb="000284C7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00134074"/>
         <bgColor rgb="00134074"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="000284C7"/>
-        <bgColor rgb="000284C7"/>
+        <fgColor rgb="00F0F9FF"/>
+        <bgColor rgb="00F0F9FF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F8FAFC"/>
         <bgColor rgb="00F8FAFC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F0F9FF"/>
-        <bgColor rgb="00F0F9FF"/>
       </patternFill>
     </fill>
     <fill>
@@ -148,52 +148,47 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -560,18 +555,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J54"/>
+  <dimension ref="A1:K54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="54" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="4" customWidth="1" min="8" max="8"/>
     <col width="30" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="4" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -580,324 +577,302 @@
           <t>MAPA DE CARRERA | PROFESORADO DE PSICOLOGÍA</t>
         </is>
       </c>
-    </row>
-    <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>CONTROL DE TRAYECTORIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>La Caravana + Estudiantes Independientes | Altillo JVG - ISP Joaquín V. González</t>
         </is>
       </c>
-    </row>
-    <row r="3" ht="28" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Asignatura / Materia</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>¿Cursada Regular? (SI/NO)</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>¿Final Aprobado? (SI/NO)</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Régimen / Año</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>¿Cursada?</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>¿Final?</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>Estado de Avance</t>
-        </is>
-      </c>
+      <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>Total de Materias del Plan</t>
+        </is>
+      </c>
+      <c r="J2" s="5" t="n">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>📊 RESUMEN DE AVANCE</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
+          <t>Materias con Cursada Regular</t>
+        </is>
+      </c>
+      <c r="J3" s="5">
+        <f>COUNTIF(B6:B54, "SI")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Materia / Asignatura Oficial</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Cursada Regular</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Final Aprobado</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Año / Tramo</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Condición Cursada</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>Condición Final</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>Estado General</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>Finales / Materias Aprobadas</t>
+        </is>
+      </c>
+      <c r="J4" s="5">
+        <f>COUNTIF(C6:C54, "SI")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>📌 1° AÑO</t>
         </is>
       </c>
-      <c r="I4" s="6" t="inlineStr">
-        <is>
-          <t>Total Materias del Plan</t>
-        </is>
-      </c>
-      <c r="J4" s="7" t="n">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="5" ht="24" customHeight="1">
-      <c r="A5" s="8" t="inlineStr">
-        <is>
-          <t>ANTROPOLOGIA SOCIAL Y CULTURAL</t>
-        </is>
-      </c>
-      <c r="B5" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="C5" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D5" s="10" t="inlineStr">
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>Finales Adeudados</t>
+        </is>
+      </c>
+      <c r="J5" s="5">
+        <f>COUNTIF(F6:F54, "ADEUDA FINAL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>Antropologia Social y Cultural</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="inlineStr">
         <is>
           <t>1° Año</t>
         </is>
       </c>
-      <c r="E5" s="9">
-        <f>IF(OR(B5="SI",B5="SÍ",B5=TRUE),"REGULAR","PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F5" s="9">
-        <f>IF(OR(C5="SI",C5="SÍ",C5=TRUE),"APROBADA",IF(OR(B5="SI",B5="SÍ",B5=TRUE),"RINDE FINAL","ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G5" s="9">
-        <f>IF(OR(C5="SI",C5="SÍ",C5=TRUE),"✅ Aprobada",IF(OR(B5="SI",B5="SÍ",B5=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
-        <v/>
-      </c>
-      <c r="I5" s="6" t="inlineStr">
-        <is>
-          <t>Cursadas Regulares</t>
-        </is>
-      </c>
-      <c r="J5" s="7">
-        <f>COUNTIF(B4:B54, "S*") + COUNTIF(B4:B54, TRUE)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="11" t="inlineStr">
-        <is>
-          <t>BIOLOGIA (1° CUATRIMESTRE)</t>
-        </is>
-      </c>
-      <c r="B6" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="C6" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D6" s="12" t="inlineStr">
+      <c r="E6" s="10">
+        <f>IF(B6="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F6" s="10">
+        <f>IF(C6="SI", "APROBADO", IF(B6="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G6" s="11">
+        <f>IF(C6="SI", "🟢 Aprobada", IF(B6="SI", "🟡 Regular", "🟣 Pendiente"))</f>
+        <v/>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>% Cursadas Completadas</t>
+        </is>
+      </c>
+      <c r="J6" s="12">
+        <f>COUNTIF(B6:B54, "SI")/44</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>Biología</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr">
         <is>
           <t>1° Año</t>
         </is>
       </c>
-      <c r="E6" s="9">
-        <f>IF(OR(B6="SI",B6="SÍ",B6=TRUE),"REGULAR","PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F6" s="9">
-        <f>IF(OR(C6="SI",C6="SÍ",C6=TRUE),"APROBADA",IF(OR(B6="SI",B6="SÍ",B6=TRUE),"RINDE FINAL","ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G6" s="9">
-        <f>IF(OR(C6="SI",C6="SÍ",C6=TRUE),"✅ Aprobada",IF(OR(B6="SI",B6="SÍ",B6=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
-        <v/>
-      </c>
-      <c r="I6" s="6" t="inlineStr">
-        <is>
-          <t>Finales Aprobados</t>
-        </is>
-      </c>
-      <c r="J6" s="7">
-        <f>COUNTIF(C4:C54, "S*") + COUNTIF(C4:C54, TRUE)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="8" t="inlineStr">
-        <is>
-          <t>FILOSOFIA</t>
-        </is>
-      </c>
-      <c r="B7" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="C7" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D7" s="10" t="inlineStr">
+      <c r="E7" s="10">
+        <f>IF(B7="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F7" s="10">
+        <f>IF(C7="SI", "APROBADO", IF(B7="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G7" s="11">
+        <f>IF(C7="SI", "🟢 Aprobada", IF(B7="SI", "🟡 Regular", "🟣 Pendiente"))</f>
+        <v/>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>% Carrera Aprobada (Finales)</t>
+        </is>
+      </c>
+      <c r="J7" s="12">
+        <f>COUNTIF(C6:C54, "SI")/44</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>Filosofía</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="inlineStr">
         <is>
           <t>1° Año</t>
         </is>
       </c>
-      <c r="E7" s="9">
-        <f>IF(OR(B7="SI",B7="SÍ",B7=TRUE),"REGULAR","PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F7" s="9">
-        <f>IF(OR(C7="SI",C7="SÍ",C7=TRUE),"APROBADA",IF(OR(B7="SI",B7="SÍ",B7=TRUE),"RINDE FINAL","ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G7" s="9">
-        <f>IF(OR(C7="SI",C7="SÍ",C7=TRUE),"✅ Aprobada",IF(OR(B7="SI",B7="SÍ",B7=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
-        <v/>
-      </c>
-      <c r="I7" s="6" t="inlineStr">
-        <is>
-          <t>Finales Adeudados</t>
-        </is>
-      </c>
-      <c r="J7" s="7">
-        <f>J5-J6</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="11" t="inlineStr">
-        <is>
-          <t>LECTURA, ESCRITURA Y ORALIDAD I</t>
-        </is>
-      </c>
-      <c r="B8" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="C8" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D8" s="12" t="inlineStr">
+      <c r="E8" s="10">
+        <f>IF(B8="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F8" s="10">
+        <f>IF(C8="SI", "APROBADO", IF(B8="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G8" s="11">
+        <f>IF(C8="SI", "🟢 Aprobada", IF(B8="SI", "🟡 Regular", "🟣 Pendiente"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>Lectura, Escritura y Oralidad I (LEO 1)</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
         <is>
           <t>1° Año</t>
         </is>
       </c>
-      <c r="E8" s="9">
-        <f>IF(OR(B8="SI",B8="SÍ",B8=TRUE),"REGULAR","PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F8" s="9">
-        <f>IF(OR(C8="SI",C8="SÍ",C8=TRUE),"APROBADA",IF(OR(B8="SI",B8="SÍ",B8=TRUE),"RINDE FINAL","ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G8" s="9">
-        <f>IF(OR(C8="SI",C8="SÍ",C8=TRUE),"✅ Aprobada",IF(OR(B8="SI",B8="SÍ",B8=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
-        <v/>
-      </c>
-      <c r="I8" s="6" t="inlineStr">
-        <is>
-          <t>% Cursadas Completadas</t>
-        </is>
-      </c>
-      <c r="J8" s="13">
-        <f>J5/45</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>LOGICA (1° Cuat.)</t>
-        </is>
-      </c>
-      <c r="B9" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="C9" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D9" s="10" t="inlineStr">
+      <c r="E9" s="10">
+        <f>IF(B9="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F9" s="10">
+        <f>IF(C9="SI", "APROBADO", IF(B9="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G9" s="11">
+        <f>IF(C9="SI", "🟢 Aprobada", IF(B9="SI", "🟡 Regular", "🟣 Pendiente"))</f>
+        <v/>
+      </c>
+      <c r="I9" s="13" t="inlineStr">
+        <is>
+          <t>INSTRUCCIONES DE USO</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>Logica</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="inlineStr">
         <is>
           <t>1° Año</t>
         </is>
       </c>
-      <c r="E9" s="9">
-        <f>IF(OR(B9="SI",B9="SÍ",B9=TRUE),"REGULAR","PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F9" s="9">
-        <f>IF(OR(C9="SI",C9="SÍ",C9=TRUE),"APROBADA",IF(OR(B9="SI",B9="SÍ",B9=TRUE),"RINDE FINAL","ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G9" s="9">
-        <f>IF(OR(C9="SI",C9="SÍ",C9=TRUE),"✅ Aprobada",IF(OR(B9="SI",B9="SÍ",B9=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
-        <v/>
-      </c>
-      <c r="I9" s="6" t="inlineStr">
-        <is>
-          <t>% Carrera Aprobada (Finales)</t>
-        </is>
-      </c>
-      <c r="J9" s="13">
-        <f>J6/45</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="11" t="inlineStr">
-        <is>
-          <t>METODOLOGIA DE LA INV.SOCIAL (1° Cuatr.)</t>
-        </is>
-      </c>
-      <c r="B10" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="C10" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D10" s="12" t="inlineStr">
-        <is>
-          <t>1° Año</t>
-        </is>
-      </c>
-      <c r="E10" s="9">
-        <f>IF(OR(B10="SI",B10="SÍ",B10=TRUE),"REGULAR","PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F10" s="9">
-        <f>IF(OR(C10="SI",C10="SÍ",C10=TRUE),"APROBADA",IF(OR(B10="SI",B10="SÍ",B10=TRUE),"RINDE FINAL","ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G10" s="9">
-        <f>IF(OR(C10="SI",C10="SÍ",C10=TRUE),"✅ Aprobada",IF(OR(B10="SI",B10="SÍ",B10=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
-        <v/>
+      <c r="E10" s="10">
+        <f>IF(B10="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F10" s="10">
+        <f>IF(C10="SI", "APROBADO", IF(B10="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G10" s="11">
+        <f>IF(C10="SI", "🟢 Aprobada", IF(B10="SI", "🟡 Regular", "🟣 Pendiente"))</f>
+        <v/>
+      </c>
+      <c r="I10" s="14" t="inlineStr">
+        <is>
+          <t>1. Hace clic en la celda y elegi 'SI' o 'NO' desde el menu desplegable.</t>
+        </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>PEDAGOGIA</t>
+          <t>METODOLOGIA DE LA INV.SOCIAL (1° Cuatr.)</t>
         </is>
       </c>
       <c r="B11" s="9" t="inlineStr">
@@ -915,28 +890,28 @@
           <t>1° Año</t>
         </is>
       </c>
-      <c r="E11" s="9">
-        <f>IF(OR(B11="SI",B11="SÍ",B11=TRUE),"REGULAR","PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F11" s="9">
-        <f>IF(OR(C11="SI",C11="SÍ",C11=TRUE),"APROBADA",IF(OR(B11="SI",B11="SÍ",B11=TRUE),"RINDE FINAL","ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G11" s="9">
-        <f>IF(OR(C11="SI",C11="SÍ",C11=TRUE),"✅ Aprobada",IF(OR(B11="SI",B11="SÍ",B11=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
+      <c r="E11" s="10">
+        <f>IF(B11="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F11" s="10">
+        <f>IF(C11="SI", "APROBADO", IF(B11="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G11" s="11">
+        <f>IF(C11="SI", "🟢 Aprobada", IF(B11="SI", "🟡 Regular", "🟣 Pendiente"))</f>
         <v/>
       </c>
       <c r="I11" s="14" t="inlineStr">
         <is>
-          <t>💡 INSTRUCCIONES DE USO</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="26" customHeight="1">
-      <c r="A12" s="11" t="inlineStr">
-        <is>
-          <t>PROC. COLECTIVOS Y PROBLEMAS SOCIALES</t>
+          <t>2. Columna B: Marca 'SI' si tenes la cursada regular aprobada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>Pedagogía</t>
         </is>
       </c>
       <c r="B12" s="9" t="inlineStr">
@@ -949,33 +924,33 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D12" s="12" t="inlineStr">
+      <c r="D12" s="10" t="inlineStr">
         <is>
           <t>1° Año</t>
         </is>
       </c>
-      <c r="E12" s="9">
-        <f>IF(OR(B12="SI",B12="SÍ",B12=TRUE),"REGULAR","PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F12" s="9">
-        <f>IF(OR(C12="SI",C12="SÍ",C12=TRUE),"APROBADA",IF(OR(B12="SI",B12="SÍ",B12=TRUE),"RINDE FINAL","ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G12" s="9">
-        <f>IF(OR(C12="SI",C12="SÍ",C12=TRUE),"✅ Aprobada",IF(OR(B12="SI",B12="SÍ",B12=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
-        <v/>
-      </c>
-      <c r="I12" s="15" t="inlineStr">
-        <is>
-          <t>1. Hacé clic en la celda y elegí 'SI' o 'NO' desde el menú desplegable.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="26" customHeight="1">
+      <c r="E12" s="10">
+        <f>IF(B12="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F12" s="10">
+        <f>IF(C12="SI", "APROBADO", IF(B12="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G12" s="11">
+        <f>IF(C12="SI", "🟢 Aprobada", IF(B12="SI", "🟡 Regular", "🟣 Pendiente"))</f>
+        <v/>
+      </c>
+      <c r="I12" s="14" t="inlineStr">
+        <is>
+          <t>3. Columna C: Marca 'SI' si aprobaste el final o promocionaste.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>PSICOLOGIA GENERAL</t>
+          <t>Proc. Colectivos y Problemas Sociales</t>
         </is>
       </c>
       <c r="B13" s="9" t="inlineStr">
@@ -993,28 +968,28 @@
           <t>1° Año</t>
         </is>
       </c>
-      <c r="E13" s="9">
-        <f>IF(OR(B13="SI",B13="SÍ",B13=TRUE),"REGULAR","PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F13" s="9">
-        <f>IF(OR(C13="SI",C13="SÍ",C13=TRUE),"APROBADA",IF(OR(B13="SI",B13="SÍ",B13=TRUE),"RINDE FINAL","ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G13" s="9">
-        <f>IF(OR(C13="SI",C13="SÍ",C13=TRUE),"✅ Aprobada",IF(OR(B13="SI",B13="SÍ",B13=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
-        <v/>
-      </c>
-      <c r="I13" s="15" t="inlineStr">
-        <is>
-          <t>2. Columna B: Marcá 'SI' si tenés la cursada regular aprobada.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="26" customHeight="1">
-      <c r="A14" s="11" t="inlineStr">
-        <is>
-          <t>TRABAJO DE CAMPO I</t>
+      <c r="E13" s="10">
+        <f>IF(B13="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F13" s="10">
+        <f>IF(C13="SI", "APROBADO", IF(B13="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G13" s="11">
+        <f>IF(C13="SI", "🟢 Aprobada", IF(B13="SI", "🟡 Regular", "🟣 Pendiente"))</f>
+        <v/>
+      </c>
+      <c r="I13" s="14" t="inlineStr">
+        <is>
+          <t>4. Las columnas E, F y G se actualizan automaticamente en tiempo real.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>Psicología GENERAL</t>
         </is>
       </c>
       <c r="B14" s="9" t="inlineStr">
@@ -1027,157 +1002,147 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D14" s="12" t="inlineStr">
+      <c r="D14" s="10" t="inlineStr">
         <is>
           <t>1° Año</t>
         </is>
       </c>
-      <c r="E14" s="9">
-        <f>IF(OR(B14="SI",B14="SÍ",B14=TRUE),"REGULAR","PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F14" s="9">
-        <f>IF(OR(C14="SI",C14="SÍ",C14=TRUE),"APROBADA",IF(OR(B14="SI",B14="SÍ",B14=TRUE),"RINDE FINAL","ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G14" s="9">
-        <f>IF(OR(C14="SI",C14="SÍ",C14=TRUE),"✅ Aprobada",IF(OR(B14="SI",B14="SÍ",B14=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
-        <v/>
-      </c>
-      <c r="I14" s="15" t="inlineStr">
-        <is>
-          <t>3. Columna C: Marcá 'SI' si aprobaste el final o promocionaste.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="26" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
+      <c r="E14" s="10">
+        <f>IF(B14="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F14" s="10">
+        <f>IF(C14="SI", "APROBADO", IF(B14="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G14" s="11">
+        <f>IF(C14="SI", "🟢 Aprobada", IF(B14="SI", "🟡 Regular", "🟣 Pendiente"))</f>
+        <v/>
+      </c>
+      <c r="I14" s="14" t="inlineStr">
+        <is>
+          <t>5. El panel lateral calcula tu avance y porcentaje de carrera en vivo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>Trabajo de Campo I</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="inlineStr">
+        <is>
+          <t>1° Año</t>
+        </is>
+      </c>
+      <c r="E15" s="10">
+        <f>IF(B15="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F15" s="10">
+        <f>IF(C15="SI", "APROBADO", IF(B15="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G15" s="11">
+        <f>IF(C15="SI", "🟢 Aprobada", IF(B15="SI", "🟡 Regular", "🟣 Pendiente"))</f>
+        <v/>
+      </c>
+      <c r="I15" s="14" t="inlineStr">
+        <is>
+          <t>6. Podes subir el archivo a tu Google Drive personal para editarlo online.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="7" t="inlineStr">
         <is>
           <t>📌 2° AÑO</t>
         </is>
       </c>
-      <c r="I15" s="15" t="inlineStr">
-        <is>
-          <t>4. Las columnas E, F y G se actualizan automáticamente en tiempo real.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="26" customHeight="1">
-      <c r="A16" s="11" t="inlineStr">
-        <is>
-          <t>APROX. AL PROCESO SALUD-ENFERMEDAD(1° CUATR.)</t>
-        </is>
-      </c>
-      <c r="B16" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="C16" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D16" s="12" t="inlineStr">
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>Aprox. al Proceso Salud-enfermedad(1° Cuatr.)</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D17" s="10" t="inlineStr">
         <is>
           <t>2° Año</t>
         </is>
       </c>
-      <c r="E16" s="9">
-        <f>IF(OR(B16="SI",B16="SÍ",B16=TRUE),"REGULAR","PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F16" s="9">
-        <f>IF(OR(C16="SI",C16="SÍ",C16=TRUE),"APROBADA",IF(OR(B16="SI",B16="SÍ",B16=TRUE),"RINDE FINAL","ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G16" s="9">
-        <f>IF(OR(C16="SI",C16="SÍ",C16=TRUE),"✅ Aprobada",IF(OR(B16="SI",B16="SÍ",B16=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
-        <v/>
-      </c>
-      <c r="I16" s="15" t="inlineStr">
-        <is>
-          <t>5. El panel lateral calcula tu avance y porcentaje de carrera en vivo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="26" customHeight="1">
-      <c r="A17" s="8" t="inlineStr">
-        <is>
-          <t>BASES NEUROFISIOLÓGICAS "A"</t>
-        </is>
-      </c>
-      <c r="B17" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="C17" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D17" s="10" t="inlineStr">
+      <c r="E17" s="10">
+        <f>IF(B17="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F17" s="10">
+        <f>IF(C17="SI", "APROBADO", IF(B17="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G17" s="11">
+        <f>IF(C17="SI", "🟢 Aprobada", IF(B17="SI", "🟡 Regular", "🟣 Pendiente"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>Bases Neurofisiológicas</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="D18" s="10" t="inlineStr">
         <is>
           <t>2° Año</t>
         </is>
       </c>
-      <c r="E17" s="9">
-        <f>IF(OR(B17="SI",B17="SÍ",B17=TRUE),"REGULAR","PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F17" s="9">
-        <f>IF(OR(C17="SI",C17="SÍ",C17=TRUE),"APROBADA",IF(OR(B17="SI",B17="SÍ",B17=TRUE),"RINDE FINAL","ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G17" s="9">
-        <f>IF(OR(C17="SI",C17="SÍ",C17=TRUE),"✅ Aprobada",IF(OR(B17="SI",B17="SÍ",B17=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
-        <v/>
-      </c>
-      <c r="I17" s="15" t="inlineStr">
-        <is>
-          <t>6. Podés subir el archivo a tu Google Drive personal para editarlo online.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="11" t="inlineStr">
-        <is>
-          <t>DIDACTICA GENERAL</t>
-        </is>
-      </c>
-      <c r="B18" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="C18" s="9" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="D18" s="12" t="inlineStr">
-        <is>
-          <t>2° Año</t>
-        </is>
-      </c>
-      <c r="E18" s="9">
-        <f>IF(OR(B18="SI",B18="SÍ",B18=TRUE),"REGULAR","PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F18" s="9">
-        <f>IF(OR(C18="SI",C18="SÍ",C18=TRUE),"APROBADA",IF(OR(B18="SI",B18="SÍ",B18=TRUE),"RINDE FINAL","ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G18" s="9">
-        <f>IF(OR(C18="SI",C18="SÍ",C18=TRUE),"✅ Aprobada",IF(OR(B18="SI",B18="SÍ",B18=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
+      <c r="E18" s="10">
+        <f>IF(B18="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F18" s="10">
+        <f>IF(C18="SI", "APROBADO", IF(B18="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G18" s="11">
+        <f>IF(C18="SI", "🟢 Aprobada", IF(B18="SI", "🟡 Regular", "🟣 Pendiente"))</f>
         <v/>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>EPISTEMOLOGIA GRAL Y ESPECIAL</t>
+          <t>Didáctica GENERAL</t>
         </is>
       </c>
       <c r="B19" s="9" t="inlineStr">
@@ -1195,23 +1160,23 @@
           <t>2° Año</t>
         </is>
       </c>
-      <c r="E19" s="9">
-        <f>IF(OR(B19="SI",B19="SÍ",B19=TRUE),"REGULAR","PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F19" s="9">
-        <f>IF(OR(C19="SI",C19="SÍ",C19=TRUE),"APROBADA",IF(OR(B19="SI",B19="SÍ",B19=TRUE),"RINDE FINAL","ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G19" s="9">
-        <f>IF(OR(C19="SI",C19="SÍ",C19=TRUE),"✅ Aprobada",IF(OR(B19="SI",B19="SÍ",B19=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
+      <c r="E19" s="10">
+        <f>IF(B19="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F19" s="10">
+        <f>IF(C19="SI", "APROBADO", IF(B19="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G19" s="11">
+        <f>IF(C19="SI", "🟢 Aprobada", IF(B19="SI", "🟡 Regular", "🟣 Pendiente"))</f>
         <v/>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="11" t="inlineStr">
-        <is>
-          <t>ESTADO, SOCIEDAD Y DD HH</t>
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>Epistemologia Gral y Especial</t>
         </is>
       </c>
       <c r="B20" s="9" t="inlineStr">
@@ -1224,28 +1189,28 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D20" s="12" t="inlineStr">
+      <c r="D20" s="10" t="inlineStr">
         <is>
           <t>2° Año</t>
         </is>
       </c>
-      <c r="E20" s="9">
-        <f>IF(OR(B20="SI",B20="SÍ",B20=TRUE),"REGULAR","PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F20" s="9">
-        <f>IF(OR(C20="SI",C20="SÍ",C20=TRUE),"APROBADA",IF(OR(B20="SI",B20="SÍ",B20=TRUE),"RINDE FINAL","ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G20" s="9">
-        <f>IF(OR(C20="SI",C20="SÍ",C20=TRUE),"✅ Aprobada",IF(OR(B20="SI",B20="SÍ",B20=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
+      <c r="E20" s="10">
+        <f>IF(B20="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F20" s="10">
+        <f>IF(C20="SI", "APROBADO", IF(B20="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G20" s="11">
+        <f>IF(C20="SI", "🟢 Aprobada", IF(B20="SI", "🟡 Regular", "🟣 Pendiente"))</f>
         <v/>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>LECTURA, ESCRITURA Y ORALIDAD II</t>
+          <t>ESTADO, SOCIEDAD Y Derechos Humanos</t>
         </is>
       </c>
       <c r="B21" s="9" t="inlineStr">
@@ -1263,21 +1228,21 @@
           <t>2° Año</t>
         </is>
       </c>
-      <c r="E21" s="9">
-        <f>IF(OR(B21="SI",B21="SÍ",B21=TRUE),"REGULAR","PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F21" s="9">
-        <f>IF(OR(C21="SI",C21="SÍ",C21=TRUE),"APROBADA",IF(OR(B21="SI",B21="SÍ",B21=TRUE),"RINDE FINAL","ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G21" s="9">
-        <f>IF(OR(C21="SI",C21="SÍ",C21=TRUE),"✅ Aprobada",IF(OR(B21="SI",B21="SÍ",B21=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
+      <c r="E21" s="10">
+        <f>IF(B21="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F21" s="10">
+        <f>IF(C21="SI", "APROBADO", IF(B21="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G21" s="11">
+        <f>IF(C21="SI", "🟢 Aprobada", IF(B21="SI", "🟡 Regular", "🟣 Pendiente"))</f>
         <v/>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="11" t="inlineStr">
+      <c r="A22" s="8" t="inlineStr">
         <is>
           <t>NUEVAS TECNOLOGIAS (Cuatrimestral)</t>
         </is>
@@ -1292,28 +1257,28 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D22" s="12" t="inlineStr">
+      <c r="D22" s="10" t="inlineStr">
         <is>
           <t>2° Año</t>
         </is>
       </c>
-      <c r="E22" s="9">
-        <f>IF(OR(B22="SI",B22="SÍ",B22=TRUE),"REGULAR","PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F22" s="9">
-        <f>IF(OR(C22="SI",C22="SÍ",C22=TRUE),"APROBADA",IF(OR(B22="SI",B22="SÍ",B22=TRUE),"RINDE FINAL","ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G22" s="9">
-        <f>IF(OR(C22="SI",C22="SÍ",C22=TRUE),"✅ Aprobada",IF(OR(B22="SI",B22="SÍ",B22=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
+      <c r="E22" s="10">
+        <f>IF(B22="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F22" s="10">
+        <f>IF(C22="SI", "APROBADO", IF(B22="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G22" s="11">
+        <f>IF(C22="SI", "🟢 Aprobada", IF(B22="SI", "🟡 Regular", "🟣 Pendiente"))</f>
         <v/>
       </c>
     </row>
     <row r="23" ht="20" customHeight="1">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>PSICOLOGIA DE LOS CICLOS VITALES I</t>
+          <t>Psicología DE LOS CICLOS VITALES I</t>
         </is>
       </c>
       <c r="B23" s="9" t="inlineStr">
@@ -1331,23 +1296,23 @@
           <t>2° Año</t>
         </is>
       </c>
-      <c r="E23" s="9">
-        <f>IF(OR(B23="SI",B23="SÍ",B23=TRUE),"REGULAR","PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F23" s="9">
-        <f>IF(OR(C23="SI",C23="SÍ",C23=TRUE),"APROBADA",IF(OR(B23="SI",B23="SÍ",B23=TRUE),"RINDE FINAL","ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G23" s="9">
-        <f>IF(OR(C23="SI",C23="SÍ",C23=TRUE),"✅ Aprobada",IF(OR(B23="SI",B23="SÍ",B23=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
+      <c r="E23" s="10">
+        <f>IF(B23="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F23" s="10">
+        <f>IF(C23="SI", "APROBADO", IF(B23="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G23" s="11">
+        <f>IF(C23="SI", "🟢 Aprobada", IF(B23="SI", "🟡 Regular", "🟣 Pendiente"))</f>
         <v/>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="11" t="inlineStr">
-        <is>
-          <t>PSICOLOGIA EDUCACIONAL</t>
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>Psicología EDUCACIONAL</t>
         </is>
       </c>
       <c r="B24" s="9" t="inlineStr">
@@ -1360,28 +1325,28 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D24" s="12" t="inlineStr">
+      <c r="D24" s="10" t="inlineStr">
         <is>
           <t>2° Año</t>
         </is>
       </c>
-      <c r="E24" s="9">
-        <f>IF(OR(B24="SI",B24="SÍ",B24=TRUE),"REGULAR","PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F24" s="9">
-        <f>IF(OR(C24="SI",C24="SÍ",C24=TRUE),"APROBADA",IF(OR(B24="SI",B24="SÍ",B24=TRUE),"RINDE FINAL","ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G24" s="9">
-        <f>IF(OR(C24="SI",C24="SÍ",C24=TRUE),"✅ Aprobada",IF(OR(B24="SI",B24="SÍ",B24=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
+      <c r="E24" s="10">
+        <f>IF(B24="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F24" s="10">
+        <f>IF(C24="SI", "APROBADO", IF(B24="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G24" s="11">
+        <f>IF(C24="SI", "🟢 Aprobada", IF(B24="SI", "🟡 Regular", "🟣 Pendiente"))</f>
         <v/>
       </c>
     </row>
     <row r="25" ht="20" customHeight="1">
       <c r="A25" s="8" t="inlineStr">
         <is>
-          <t>PSICOLOGIA SOCIAL</t>
+          <t>Psicología SOCIAL</t>
         </is>
       </c>
       <c r="B25" s="9" t="inlineStr">
@@ -1399,23 +1364,23 @@
           <t>2° Año</t>
         </is>
       </c>
-      <c r="E25" s="9">
-        <f>IF(OR(B25="SI",B25="SÍ",B25=TRUE),"REGULAR","PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F25" s="9">
-        <f>IF(OR(C25="SI",C25="SÍ",C25=TRUE),"APROBADA",IF(OR(B25="SI",B25="SÍ",B25=TRUE),"RINDE FINAL","ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G25" s="9">
-        <f>IF(OR(C25="SI",C25="SÍ",C25=TRUE),"✅ Aprobada",IF(OR(B25="SI",B25="SÍ",B25=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
+      <c r="E25" s="10">
+        <f>IF(B25="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F25" s="10">
+        <f>IF(C25="SI", "APROBADO", IF(B25="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G25" s="11">
+        <f>IF(C25="SI", "🟢 Aprobada", IF(B25="SI", "🟡 Regular", "🟣 Pendiente"))</f>
         <v/>
       </c>
     </row>
     <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="11" t="inlineStr">
-        <is>
-          <t>TRABAJO DE CAMPO II</t>
+      <c r="A26" s="8" t="inlineStr">
+        <is>
+          <t>Trabajo de Campo II</t>
         </is>
       </c>
       <c r="B26" s="9" t="inlineStr">
@@ -1428,35 +1393,35 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D26" s="12" t="inlineStr">
+      <c r="D26" s="10" t="inlineStr">
         <is>
           <t>2° Año</t>
         </is>
       </c>
-      <c r="E26" s="9">
-        <f>IF(OR(B26="SI",B26="SÍ",B26=TRUE),"REGULAR","PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F26" s="9">
-        <f>IF(OR(C26="SI",C26="SÍ",C26=TRUE),"APROBADA",IF(OR(B26="SI",B26="SÍ",B26=TRUE),"RINDE FINAL","ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G26" s="9">
-        <f>IF(OR(C26="SI",C26="SÍ",C26=TRUE),"✅ Aprobada",IF(OR(B26="SI",B26="SÍ",B26=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27" ht="24" customHeight="1">
-      <c r="A27" s="5" t="inlineStr">
+      <c r="E26" s="10">
+        <f>IF(B26="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F26" s="10">
+        <f>IF(C26="SI", "APROBADO", IF(B26="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G26" s="11">
+        <f>IF(C26="SI", "🟢 Aprobada", IF(B26="SI", "🟡 Regular", "🟣 Pendiente"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="7" t="inlineStr">
         <is>
           <t>📌 3° AÑO</t>
         </is>
       </c>
     </row>
     <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="11" t="inlineStr">
-        <is>
-          <t>ADOLESCENCIA Y MUNDO CONT.(1° Cuat.)</t>
+      <c r="A28" s="8" t="inlineStr">
+        <is>
+          <t>Adolescencia y Mundo Cont</t>
         </is>
       </c>
       <c r="B28" s="9" t="inlineStr">
@@ -1469,28 +1434,28 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D28" s="12" t="inlineStr">
+      <c r="D28" s="10" t="inlineStr">
         <is>
           <t>3° Año</t>
         </is>
       </c>
-      <c r="E28" s="9">
-        <f>IF(OR(B28="SI",B28="SÍ",B28=TRUE),"REGULAR","PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F28" s="9">
-        <f>IF(OR(C28="SI",C28="SÍ",C28=TRUE),"APROBADA",IF(OR(B28="SI",B28="SÍ",B28=TRUE),"RINDE FINAL","ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G28" s="9">
-        <f>IF(OR(C28="SI",C28="SÍ",C28=TRUE),"✅ Aprobada",IF(OR(B28="SI",B28="SÍ",B28=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
+      <c r="E28" s="10">
+        <f>IF(B28="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F28" s="10">
+        <f>IF(C28="SI", "APROBADO", IF(B28="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G28" s="11">
+        <f>IF(C28="SI", "🟢 Aprobada", IF(B28="SI", "🟡 Regular", "🟣 Pendiente"))</f>
         <v/>
       </c>
     </row>
     <row r="29" ht="20" customHeight="1">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>ESTRATEGIAS PARA LA RES. DE CONFLICTOS(1°C)</t>
+          <t>Estrategias para la Res. de Conflictos</t>
         </is>
       </c>
       <c r="B29" s="9" t="inlineStr">
@@ -1508,23 +1473,23 @@
           <t>3° Año</t>
         </is>
       </c>
-      <c r="E29" s="9">
-        <f>IF(OR(B29="SI",B29="SÍ",B29=TRUE),"REGULAR","PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F29" s="9">
-        <f>IF(OR(C29="SI",C29="SÍ",C29=TRUE),"APROBADA",IF(OR(B29="SI",B29="SÍ",B29=TRUE),"RINDE FINAL","ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G29" s="9">
-        <f>IF(OR(C29="SI",C29="SÍ",C29=TRUE),"✅ Aprobada",IF(OR(B29="SI",B29="SÍ",B29=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
+      <c r="E29" s="10">
+        <f>IF(B29="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F29" s="10">
+        <f>IF(C29="SI", "APROBADO", IF(B29="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G29" s="11">
+        <f>IF(C29="SI", "🟢 Aprobada", IF(B29="SI", "🟡 Regular", "🟣 Pendiente"))</f>
         <v/>
       </c>
     </row>
     <row r="30" ht="20" customHeight="1">
-      <c r="A30" s="11" t="inlineStr">
-        <is>
-          <t>HISTORIA DE LA EDUCACION ARGENTINA</t>
+      <c r="A30" s="8" t="inlineStr">
+        <is>
+          <t>HISTORIA DE LA Educación ARGENTINA</t>
         </is>
       </c>
       <c r="B30" s="9" t="inlineStr">
@@ -1537,28 +1502,28 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D30" s="12" t="inlineStr">
+      <c r="D30" s="10" t="inlineStr">
         <is>
           <t>3° Año</t>
         </is>
       </c>
-      <c r="E30" s="9">
-        <f>IF(OR(B30="SI",B30="SÍ",B30=TRUE),"REGULAR","PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F30" s="9">
-        <f>IF(OR(C30="SI",C30="SÍ",C30=TRUE),"APROBADA",IF(OR(B30="SI",B30="SÍ",B30=TRUE),"RINDE FINAL","ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G30" s="9">
-        <f>IF(OR(C30="SI",C30="SÍ",C30=TRUE),"✅ Aprobada",IF(OR(B30="SI",B30="SÍ",B30=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
+      <c r="E30" s="10">
+        <f>IF(B30="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F30" s="10">
+        <f>IF(C30="SI", "APROBADO", IF(B30="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G30" s="11">
+        <f>IF(C30="SI", "🟢 Aprobada", IF(B30="SI", "🟡 Regular", "🟣 Pendiente"))</f>
         <v/>
       </c>
     </row>
     <row r="31" ht="20" customHeight="1">
       <c r="A31" s="8" t="inlineStr">
         <is>
-          <t>PSICOLOGIA DE LOS CICLOS VITALES II</t>
+          <t>Psicología DE LOS CICLOS VITALES II</t>
         </is>
       </c>
       <c r="B31" s="9" t="inlineStr">
@@ -1576,23 +1541,23 @@
           <t>3° Año</t>
         </is>
       </c>
-      <c r="E31" s="9">
-        <f>IF(OR(B31="SI",B31="SÍ",B31=TRUE),"REGULAR","PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F31" s="9">
-        <f>IF(OR(C31="SI",C31="SÍ",C31=TRUE),"APROBADA",IF(OR(B31="SI",B31="SÍ",B31=TRUE),"RINDE FINAL","ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G31" s="9">
-        <f>IF(OR(C31="SI",C31="SÍ",C31=TRUE),"✅ Aprobada",IF(OR(B31="SI",B31="SÍ",B31=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
+      <c r="E31" s="10">
+        <f>IF(B31="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F31" s="10">
+        <f>IF(C31="SI", "APROBADO", IF(B31="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G31" s="11">
+        <f>IF(C31="SI", "🟢 Aprobada", IF(B31="SI", "🟡 Regular", "🟣 Pendiente"))</f>
         <v/>
       </c>
     </row>
     <row r="32" ht="20" customHeight="1">
-      <c r="A32" s="11" t="inlineStr">
-        <is>
-          <t>TECNICAS DE EXPLORACION PSICOLOGICA</t>
+      <c r="A32" s="8" t="inlineStr">
+        <is>
+          <t>Tecnicas de Exploracion Psicologica</t>
         </is>
       </c>
       <c r="B32" s="9" t="inlineStr">
@@ -1605,28 +1570,28 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D32" s="12" t="inlineStr">
+      <c r="D32" s="10" t="inlineStr">
         <is>
           <t>3° Año</t>
         </is>
       </c>
-      <c r="E32" s="9">
-        <f>IF(OR(B32="SI",B32="SÍ",B32=TRUE),"REGULAR","PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F32" s="9">
-        <f>IF(OR(C32="SI",C32="SÍ",C32=TRUE),"APROBADA",IF(OR(B32="SI",B32="SÍ",B32=TRUE),"RINDE FINAL","ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G32" s="9">
-        <f>IF(OR(C32="SI",C32="SÍ",C32=TRUE),"✅ Aprobada",IF(OR(B32="SI",B32="SÍ",B32=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
+      <c r="E32" s="10">
+        <f>IF(B32="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F32" s="10">
+        <f>IF(C32="SI", "APROBADO", IF(B32="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G32" s="11">
+        <f>IF(C32="SI", "🟢 Aprobada", IF(B32="SI", "🟡 Regular", "🟣 Pendiente"))</f>
         <v/>
       </c>
     </row>
     <row r="33" ht="20" customHeight="1">
       <c r="A33" s="8" t="inlineStr">
         <is>
-          <t>TEORIA DE LAS ORGANIZ. Y ANALISIS INST.</t>
+          <t>Teoría DE LAS ORGANIZ. Y Análisis INST</t>
         </is>
       </c>
       <c r="B33" s="9" t="inlineStr">
@@ -1644,23 +1609,23 @@
           <t>3° Año</t>
         </is>
       </c>
-      <c r="E33" s="9">
-        <f>IF(OR(B33="SI",B33="SÍ",B33=TRUE),"REGULAR","PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F33" s="9">
-        <f>IF(OR(C33="SI",C33="SÍ",C33=TRUE),"APROBADA",IF(OR(B33="SI",B33="SÍ",B33=TRUE),"RINDE FINAL","ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G33" s="9">
-        <f>IF(OR(C33="SI",C33="SÍ",C33=TRUE),"✅ Aprobada",IF(OR(B33="SI",B33="SÍ",B33=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
+      <c r="E33" s="10">
+        <f>IF(B33="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F33" s="10">
+        <f>IF(C33="SI", "APROBADO", IF(B33="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G33" s="11">
+        <f>IF(C33="SI", "🟢 Aprobada", IF(B33="SI", "🟡 Regular", "🟣 Pendiente"))</f>
         <v/>
       </c>
     </row>
     <row r="34" ht="20" customHeight="1">
-      <c r="A34" s="11" t="inlineStr">
-        <is>
-          <t>TEORIA PSICOANALITICA</t>
+      <c r="A34" s="8" t="inlineStr">
+        <is>
+          <t>Teoría PSICOANALITICA</t>
         </is>
       </c>
       <c r="B34" s="9" t="inlineStr">
@@ -1673,28 +1638,28 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D34" s="12" t="inlineStr">
+      <c r="D34" s="10" t="inlineStr">
         <is>
           <t>3° Año</t>
         </is>
       </c>
-      <c r="E34" s="9">
-        <f>IF(OR(B34="SI",B34="SÍ",B34=TRUE),"REGULAR","PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F34" s="9">
-        <f>IF(OR(C34="SI",C34="SÍ",C34=TRUE),"APROBADA",IF(OR(B34="SI",B34="SÍ",B34=TRUE),"RINDE FINAL","ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G34" s="9">
-        <f>IF(OR(C34="SI",C34="SÍ",C34=TRUE),"✅ Aprobada",IF(OR(B34="SI",B34="SÍ",B34=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
+      <c r="E34" s="10">
+        <f>IF(B34="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F34" s="10">
+        <f>IF(C34="SI", "APROBADO", IF(B34="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G34" s="11">
+        <f>IF(C34="SI", "🟢 Aprobada", IF(B34="SI", "🟡 Regular", "🟣 Pendiente"))</f>
         <v/>
       </c>
     </row>
     <row r="35" ht="20" customHeight="1">
       <c r="A35" s="8" t="inlineStr">
         <is>
-          <t>TEORIA PSICOANALITICA POST FREUDIANA</t>
+          <t>Teoría PSICOANALITICA POST FREUDIANA</t>
         </is>
       </c>
       <c r="B35" s="9" t="inlineStr">
@@ -1712,23 +1677,23 @@
           <t>3° Año</t>
         </is>
       </c>
-      <c r="E35" s="9">
-        <f>IF(OR(B35="SI",B35="SÍ",B35=TRUE),"REGULAR","PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F35" s="9">
-        <f>IF(OR(C35="SI",C35="SÍ",C35=TRUE),"APROBADA",IF(OR(B35="SI",B35="SÍ",B35=TRUE),"RINDE FINAL","ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G35" s="9">
-        <f>IF(OR(C35="SI",C35="SÍ",C35=TRUE),"✅ Aprobada",IF(OR(B35="SI",B35="SÍ",B35=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
+      <c r="E35" s="10">
+        <f>IF(B35="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F35" s="10">
+        <f>IF(C35="SI", "APROBADO", IF(B35="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G35" s="11">
+        <f>IF(C35="SI", "🟢 Aprobada", IF(B35="SI", "🟡 Regular", "🟣 Pendiente"))</f>
         <v/>
       </c>
     </row>
     <row r="36" ht="20" customHeight="1">
-      <c r="A36" s="11" t="inlineStr">
-        <is>
-          <t>TEORÍA Y PRÁCTICA DE LA COMUNIC. (1° CUATR.)</t>
+      <c r="A36" s="8" t="inlineStr">
+        <is>
+          <t>Teoría y Práctica de la Comunic. (1° Cuatr.)</t>
         </is>
       </c>
       <c r="B36" s="9" t="inlineStr">
@@ -1741,35 +1706,35 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D36" s="12" t="inlineStr">
+      <c r="D36" s="10" t="inlineStr">
         <is>
           <t>3° Año</t>
         </is>
       </c>
-      <c r="E36" s="9">
-        <f>IF(OR(B36="SI",B36="SÍ",B36=TRUE),"REGULAR","PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F36" s="9">
-        <f>IF(OR(C36="SI",C36="SÍ",C36=TRUE),"APROBADA",IF(OR(B36="SI",B36="SÍ",B36=TRUE),"RINDE FINAL","ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G36" s="9">
-        <f>IF(OR(C36="SI",C36="SÍ",C36=TRUE),"✅ Aprobada",IF(OR(B36="SI",B36="SÍ",B36=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37" ht="24" customHeight="1">
-      <c r="A37" s="5" t="inlineStr">
+      <c r="E36" s="10">
+        <f>IF(B36="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F36" s="10">
+        <f>IF(C36="SI", "APROBADO", IF(B36="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G36" s="11">
+        <f>IF(C36="SI", "🟢 Aprobada", IF(B36="SI", "🟡 Regular", "🟣 Pendiente"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37" ht="22" customHeight="1">
+      <c r="A37" s="7" t="inlineStr">
         <is>
           <t>📌 4° AÑO</t>
         </is>
       </c>
     </row>
     <row r="38" ht="20" customHeight="1">
-      <c r="A38" s="11" t="inlineStr">
-        <is>
-          <t>DIDACTICA DE LA ENS. DE LA PSICOLOGIA</t>
+      <c r="A38" s="8" t="inlineStr">
+        <is>
+          <t>Didáctica DE LA ENS. DE LA Psicología</t>
         </is>
       </c>
       <c r="B38" s="9" t="inlineStr">
@@ -1782,28 +1747,28 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D38" s="12" t="inlineStr">
+      <c r="D38" s="10" t="inlineStr">
         <is>
           <t>4° Año</t>
         </is>
       </c>
-      <c r="E38" s="9">
-        <f>IF(OR(B38="SI",B38="SÍ",B38=TRUE),"REGULAR","PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F38" s="9">
-        <f>IF(OR(C38="SI",C38="SÍ",C38=TRUE),"APROBADA",IF(OR(B38="SI",B38="SÍ",B38=TRUE),"RINDE FINAL","ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G38" s="9">
-        <f>IF(OR(C38="SI",C38="SÍ",C38=TRUE),"✅ Aprobada",IF(OR(B38="SI",B38="SÍ",B38=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
+      <c r="E38" s="10">
+        <f>IF(B38="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F38" s="10">
+        <f>IF(C38="SI", "APROBADO", IF(B38="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G38" s="11">
+        <f>IF(C38="SI", "🟢 Aprobada", IF(B38="SI", "🟡 Regular", "🟣 Pendiente"))</f>
         <v/>
       </c>
     </row>
     <row r="39" ht="20" customHeight="1">
       <c r="A39" s="8" t="inlineStr">
         <is>
-          <t>HISTORIA DE LA PSICOLOGIA (1° CUATRIMESTRE)</t>
+          <t>HISTORIA DE LA Psicología</t>
         </is>
       </c>
       <c r="B39" s="9" t="inlineStr">
@@ -1821,21 +1786,21 @@
           <t>4° Año</t>
         </is>
       </c>
-      <c r="E39" s="9">
-        <f>IF(OR(B39="SI",B39="SÍ",B39=TRUE),"REGULAR","PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F39" s="9">
-        <f>IF(OR(C39="SI",C39="SÍ",C39=TRUE),"APROBADA",IF(OR(B39="SI",B39="SÍ",B39=TRUE),"RINDE FINAL","ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G39" s="9">
-        <f>IF(OR(C39="SI",C39="SÍ",C39=TRUE),"✅ Aprobada",IF(OR(B39="SI",B39="SÍ",B39=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
+      <c r="E39" s="10">
+        <f>IF(B39="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F39" s="10">
+        <f>IF(C39="SI", "APROBADO", IF(B39="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G39" s="11">
+        <f>IF(C39="SI", "🟢 Aprobada", IF(B39="SI", "🟡 Regular", "🟣 Pendiente"))</f>
         <v/>
       </c>
     </row>
     <row r="40" ht="20" customHeight="1">
-      <c r="A40" s="11" t="inlineStr">
+      <c r="A40" s="8" t="inlineStr">
         <is>
           <t>LENGUA EXTRANJERA (Cuatrimestral)</t>
         </is>
@@ -1850,28 +1815,28 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D40" s="12" t="inlineStr">
+      <c r="D40" s="10" t="inlineStr">
         <is>
           <t>4° Año</t>
         </is>
       </c>
-      <c r="E40" s="9">
-        <f>IF(OR(B40="SI",B40="SÍ",B40=TRUE),"REGULAR","PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F40" s="9">
-        <f>IF(OR(C40="SI",C40="SÍ",C40=TRUE),"APROBADA",IF(OR(B40="SI",B40="SÍ",B40=TRUE),"RINDE FINAL","ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G40" s="9">
-        <f>IF(OR(C40="SI",C40="SÍ",C40=TRUE),"✅ Aprobada",IF(OR(B40="SI",B40="SÍ",B40=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
+      <c r="E40" s="10">
+        <f>IF(B40="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F40" s="10">
+        <f>IF(C40="SI", "APROBADO", IF(B40="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G40" s="11">
+        <f>IF(C40="SI", "🟢 Aprobada", IF(B40="SI", "🟡 Regular", "🟣 Pendiente"))</f>
         <v/>
       </c>
     </row>
     <row r="41" ht="20" customHeight="1">
       <c r="A41" s="8" t="inlineStr">
         <is>
-          <t>PRACT. DE ENS. PSICOL. N. MEDIO Y SUPERIOR</t>
+          <t>PRACT. DE ENS. PSICOL. en Nivel Medio Y SUPERIOR</t>
         </is>
       </c>
       <c r="B41" s="9" t="inlineStr">
@@ -1889,21 +1854,21 @@
           <t>4° Año</t>
         </is>
       </c>
-      <c r="E41" s="9">
-        <f>IF(OR(B41="SI",B41="SÍ",B41=TRUE),"REGULAR","PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F41" s="9">
-        <f>IF(OR(C41="SI",C41="SÍ",C41=TRUE),"APROBADA",IF(OR(B41="SI",B41="SÍ",B41=TRUE),"RINDE FINAL","ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G41" s="9">
-        <f>IF(OR(C41="SI",C41="SÍ",C41=TRUE),"✅ Aprobada",IF(OR(B41="SI",B41="SÍ",B41=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
+      <c r="E41" s="10">
+        <f>IF(B41="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F41" s="10">
+        <f>IF(C41="SI", "APROBADO", IF(B41="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G41" s="11">
+        <f>IF(C41="SI", "🟢 Aprobada", IF(B41="SI", "🟡 Regular", "🟣 Pendiente"))</f>
         <v/>
       </c>
     </row>
     <row r="42" ht="20" customHeight="1">
-      <c r="A42" s="11" t="inlineStr">
+      <c r="A42" s="8" t="inlineStr">
         <is>
           <t>PRACT.DE LA INV. PSICOLOGICA (1º CUATR.)</t>
         </is>
@@ -1918,28 +1883,28 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D42" s="12" t="inlineStr">
+      <c r="D42" s="10" t="inlineStr">
         <is>
           <t>4° Año</t>
         </is>
       </c>
-      <c r="E42" s="9">
-        <f>IF(OR(B42="SI",B42="SÍ",B42=TRUE),"REGULAR","PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F42" s="9">
-        <f>IF(OR(C42="SI",C42="SÍ",C42=TRUE),"APROBADA",IF(OR(B42="SI",B42="SÍ",B42=TRUE),"RINDE FINAL","ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G42" s="9">
-        <f>IF(OR(C42="SI",C42="SÍ",C42=TRUE),"✅ Aprobada",IF(OR(B42="SI",B42="SÍ",B42=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
+      <c r="E42" s="10">
+        <f>IF(B42="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F42" s="10">
+        <f>IF(C42="SI", "APROBADO", IF(B42="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G42" s="11">
+        <f>IF(C42="SI", "🟢 Aprobada", IF(B42="SI", "🟡 Regular", "🟣 Pendiente"))</f>
         <v/>
       </c>
     </row>
     <row r="43" ht="20" customHeight="1">
       <c r="A43" s="8" t="inlineStr">
         <is>
-          <t>PSICOLOGIA DEL ARTE (1° Cuatrim)</t>
+          <t>Psicología DEL ARTE (1° Cuatrim)</t>
         </is>
       </c>
       <c r="B43" s="9" t="inlineStr">
@@ -1957,23 +1922,23 @@
           <t>4° Año</t>
         </is>
       </c>
-      <c r="E43" s="9">
-        <f>IF(OR(B43="SI",B43="SÍ",B43=TRUE),"REGULAR","PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F43" s="9">
-        <f>IF(OR(C43="SI",C43="SÍ",C43=TRUE),"APROBADA",IF(OR(B43="SI",B43="SÍ",B43=TRUE),"RINDE FINAL","ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G43" s="9">
-        <f>IF(OR(C43="SI",C43="SÍ",C43=TRUE),"✅ Aprobada",IF(OR(B43="SI",B43="SÍ",B43=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
+      <c r="E43" s="10">
+        <f>IF(B43="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F43" s="10">
+        <f>IF(C43="SI", "APROBADO", IF(B43="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G43" s="11">
+        <f>IF(C43="SI", "🟢 Aprobada", IF(B43="SI", "🟡 Regular", "🟣 Pendiente"))</f>
         <v/>
       </c>
     </row>
     <row r="44" ht="20" customHeight="1">
-      <c r="A44" s="11" t="inlineStr">
-        <is>
-          <t>PSICOPATOLOGIA</t>
+      <c r="A44" s="8" t="inlineStr">
+        <is>
+          <t>Psicopatologia</t>
         </is>
       </c>
       <c r="B44" s="9" t="inlineStr">
@@ -1986,28 +1951,28 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D44" s="12" t="inlineStr">
+      <c r="D44" s="10" t="inlineStr">
         <is>
           <t>4° Año</t>
         </is>
       </c>
-      <c r="E44" s="9">
-        <f>IF(OR(B44="SI",B44="SÍ",B44=TRUE),"REGULAR","PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F44" s="9">
-        <f>IF(OR(C44="SI",C44="SÍ",C44=TRUE),"APROBADA",IF(OR(B44="SI",B44="SÍ",B44=TRUE),"RINDE FINAL","ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G44" s="9">
-        <f>IF(OR(C44="SI",C44="SÍ",C44=TRUE),"✅ Aprobada",IF(OR(B44="SI",B44="SÍ",B44=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
+      <c r="E44" s="10">
+        <f>IF(B44="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F44" s="10">
+        <f>IF(C44="SI", "APROBADO", IF(B44="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G44" s="11">
+        <f>IF(C44="SI", "🟢 Aprobada", IF(B44="SI", "🟡 Regular", "🟣 Pendiente"))</f>
         <v/>
       </c>
     </row>
     <row r="45" ht="20" customHeight="1">
       <c r="A45" s="8" t="inlineStr">
         <is>
-          <t>PSICOPEDAGOGIA</t>
+          <t>Psicopedagogia</t>
         </is>
       </c>
       <c r="B45" s="9" t="inlineStr">
@@ -2025,21 +1990,21 @@
           <t>4° Año</t>
         </is>
       </c>
-      <c r="E45" s="9">
-        <f>IF(OR(B45="SI",B45="SÍ",B45=TRUE),"REGULAR","PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F45" s="9">
-        <f>IF(OR(C45="SI",C45="SÍ",C45=TRUE),"APROBADA",IF(OR(B45="SI",B45="SÍ",B45=TRUE),"RINDE FINAL","ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G45" s="9">
-        <f>IF(OR(C45="SI",C45="SÍ",C45=TRUE),"✅ Aprobada",IF(OR(B45="SI",B45="SÍ",B45=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46" ht="24" customHeight="1">
-      <c r="A46" s="5" t="inlineStr">
+      <c r="E45" s="10">
+        <f>IF(B45="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F45" s="10">
+        <f>IF(C45="SI", "APROBADO", IF(B45="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G45" s="11">
+        <f>IF(C45="SI", "🟢 Aprobada", IF(B45="SI", "🟡 Regular", "🟣 Pendiente"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46" ht="22" customHeight="1">
+      <c r="A46" s="7" t="inlineStr">
         <is>
           <t>📌 5° AÑO (NIVEL SUPERIOR / TRAMO SUPERIOR)</t>
         </is>
@@ -2048,7 +2013,7 @@
     <row r="47" ht="20" customHeight="1">
       <c r="A47" s="8" t="inlineStr">
         <is>
-          <t>PEDAGOGIA DE LA CONV. ESCOLAR (1° Cuat)</t>
+          <t>Pedagogía DE LA CONV. ESCOLAR</t>
         </is>
       </c>
       <c r="B47" s="9" t="inlineStr">
@@ -2066,23 +2031,23 @@
           <t>5° Año (Nivel Superior / Tramo Superior)</t>
         </is>
       </c>
-      <c r="E47" s="9">
-        <f>IF(OR(B47="SI",B47="SÍ",B47=TRUE),"REGULAR","PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F47" s="9">
-        <f>IF(OR(C47="SI",C47="SÍ",C47=TRUE),"APROBADA",IF(OR(B47="SI",B47="SÍ",B47=TRUE),"RINDE FINAL","ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G47" s="9">
-        <f>IF(OR(C47="SI",C47="SÍ",C47=TRUE),"✅ Aprobada",IF(OR(B47="SI",B47="SÍ",B47=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
+      <c r="E47" s="10">
+        <f>IF(B47="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F47" s="10">
+        <f>IF(C47="SI", "APROBADO", IF(B47="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G47" s="11">
+        <f>IF(C47="SI", "🟢 Aprobada", IF(B47="SI", "🟡 Regular", "🟣 Pendiente"))</f>
         <v/>
       </c>
     </row>
     <row r="48" ht="20" customHeight="1">
-      <c r="A48" s="11" t="inlineStr">
-        <is>
-          <t>PRACT. DE ENS. PSICOL. N. MEDIO Y RESIDENCIA</t>
+      <c r="A48" s="8" t="inlineStr">
+        <is>
+          <t>PRACT. DE ENS. PSICOL. en Nivel Medio y Residencia</t>
         </is>
       </c>
       <c r="B48" s="9" t="inlineStr">
@@ -2095,28 +2060,28 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D48" s="12" t="inlineStr">
+      <c r="D48" s="10" t="inlineStr">
         <is>
           <t>5° Año (Nivel Superior / Tramo Superior)</t>
         </is>
       </c>
-      <c r="E48" s="9">
-        <f>IF(OR(B48="SI",B48="SÍ",B48=TRUE),"REGULAR","PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F48" s="9">
-        <f>IF(OR(C48="SI",C48="SÍ",C48=TRUE),"APROBADA",IF(OR(B48="SI",B48="SÍ",B48=TRUE),"RINDE FINAL","ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G48" s="9">
-        <f>IF(OR(C48="SI",C48="SÍ",C48=TRUE),"✅ Aprobada",IF(OR(B48="SI",B48="SÍ",B48=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
+      <c r="E48" s="10">
+        <f>IF(B48="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F48" s="10">
+        <f>IF(C48="SI", "APROBADO", IF(B48="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G48" s="11">
+        <f>IF(C48="SI", "🟢 Aprobada", IF(B48="SI", "🟡 Regular", "🟣 Pendiente"))</f>
         <v/>
       </c>
     </row>
     <row r="49" ht="20" customHeight="1">
       <c r="A49" s="8" t="inlineStr">
         <is>
-          <t>PSICOLOGIA APLICADA AL DEPORTE (1° Cuat)</t>
+          <t>Psicología APLICADA AL DEPORTE</t>
         </is>
       </c>
       <c r="B49" s="9" t="inlineStr">
@@ -2134,21 +2099,21 @@
           <t>5° Año (Nivel Superior / Tramo Superior)</t>
         </is>
       </c>
-      <c r="E49" s="9">
-        <f>IF(OR(B49="SI",B49="SÍ",B49=TRUE),"REGULAR","PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F49" s="9">
-        <f>IF(OR(C49="SI",C49="SÍ",C49=TRUE),"APROBADA",IF(OR(B49="SI",B49="SÍ",B49=TRUE),"RINDE FINAL","ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G49" s="9">
-        <f>IF(OR(C49="SI",C49="SÍ",C49=TRUE),"✅ Aprobada",IF(OR(B49="SI",B49="SÍ",B49=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50" ht="24" customHeight="1">
-      <c r="A50" s="5" t="inlineStr">
+      <c r="E49" s="10">
+        <f>IF(B49="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F49" s="10">
+        <f>IF(C49="SI", "APROBADO", IF(B49="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G49" s="11">
+        <f>IF(C49="SI", "🟢 Aprobada", IF(B49="SI", "🟡 Regular", "🟣 Pendiente"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50" ht="22" customHeight="1">
+      <c r="A50" s="7" t="inlineStr">
         <is>
           <t>📌 6° AÑO (NIVEL SUPERIOR / TRAMO SUPERIOR)</t>
         </is>
@@ -2175,21 +2140,21 @@
           <t>6° Año (Nivel Superior / Tramo Superior)</t>
         </is>
       </c>
-      <c r="E51" s="9">
-        <f>IF(OR(B51="SI",B51="SÍ",B51=TRUE),"REGULAR","PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F51" s="9">
-        <f>IF(OR(C51="SI",C51="SÍ",C51=TRUE),"APROBADA",IF(OR(B51="SI",B51="SÍ",B51=TRUE),"RINDE FINAL","ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G51" s="9">
-        <f>IF(OR(C51="SI",C51="SÍ",C51=TRUE),"✅ Aprobada",IF(OR(B51="SI",B51="SÍ",B51=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
+      <c r="E51" s="10">
+        <f>IF(B51="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F51" s="10">
+        <f>IF(C51="SI", "APROBADO", IF(B51="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G51" s="11">
+        <f>IF(C51="SI", "🟢 Aprobada", IF(B51="SI", "🟡 Regular", "🟣 Pendiente"))</f>
         <v/>
       </c>
     </row>
     <row r="52" ht="20" customHeight="1">
-      <c r="A52" s="11" t="inlineStr">
+      <c r="A52" s="8" t="inlineStr">
         <is>
           <t>Tesis / Trabajo Final de Licenciatura</t>
         </is>
@@ -2204,21 +2169,21 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D52" s="12" t="inlineStr">
+      <c r="D52" s="10" t="inlineStr">
         <is>
           <t>6° Año (Nivel Superior / Tramo Superior)</t>
         </is>
       </c>
-      <c r="E52" s="9">
-        <f>IF(OR(B52="SI",B52="SÍ",B52=TRUE),"REGULAR","PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F52" s="9">
-        <f>IF(OR(C52="SI",C52="SÍ",C52=TRUE),"APROBADA",IF(OR(B52="SI",B52="SÍ",B52=TRUE),"RINDE FINAL","ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G52" s="9">
-        <f>IF(OR(C52="SI",C52="SÍ",C52=TRUE),"✅ Aprobada",IF(OR(B52="SI",B52="SÍ",B52=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
+      <c r="E52" s="10">
+        <f>IF(B52="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F52" s="10">
+        <f>IF(C52="SI", "APROBADO", IF(B52="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G52" s="11">
+        <f>IF(C52="SI", "🟢 Aprobada", IF(B52="SI", "🟡 Regular", "🟣 Pendiente"))</f>
         <v/>
       </c>
     </row>
@@ -2243,21 +2208,21 @@
           <t>6° Año (Nivel Superior / Tramo Superior)</t>
         </is>
       </c>
-      <c r="E53" s="9">
-        <f>IF(OR(B53="SI",B53="SÍ",B53=TRUE),"REGULAR","PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F53" s="9">
-        <f>IF(OR(C53="SI",C53="SÍ",C53=TRUE),"APROBADA",IF(OR(B53="SI",B53="SÍ",B53=TRUE),"RINDE FINAL","ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G53" s="9">
-        <f>IF(OR(C53="SI",C53="SÍ",C53=TRUE),"✅ Aprobada",IF(OR(B53="SI",B53="SÍ",B53=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
+      <c r="E53" s="10">
+        <f>IF(B53="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F53" s="10">
+        <f>IF(C53="SI", "APROBADO", IF(B53="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G53" s="11">
+        <f>IF(C53="SI", "🟢 Aprobada", IF(B53="SI", "🟡 Regular", "🟣 Pendiente"))</f>
         <v/>
       </c>
     </row>
     <row r="54" ht="20" customHeight="1">
-      <c r="A54" s="11" t="inlineStr">
+      <c r="A54" s="8" t="inlineStr">
         <is>
           <t>Acreditación de Residencia Superior</t>
         </is>
@@ -2272,21 +2237,21 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="D54" s="12" t="inlineStr">
+      <c r="D54" s="10" t="inlineStr">
         <is>
           <t>6° Año (Nivel Superior / Tramo Superior)</t>
         </is>
       </c>
-      <c r="E54" s="9">
-        <f>IF(OR(B54="SI",B54="SÍ",B54=TRUE),"REGULAR","PENDIENTE")</f>
-        <v/>
-      </c>
-      <c r="F54" s="9">
-        <f>IF(OR(C54="SI",C54="SÍ",C54=TRUE),"APROBADA",IF(OR(B54="SI",B54="SÍ",B54=TRUE),"RINDE FINAL","ADEUDA"))</f>
-        <v/>
-      </c>
-      <c r="G54" s="9">
-        <f>IF(OR(C54="SI",C54="SÍ",C54=TRUE),"✅ Aprobada",IF(OR(B54="SI",B54="SÍ",B54=TRUE),"⏳ Cursada (Rinde Final)","⚪ Pendiente"))</f>
+      <c r="E54" s="10">
+        <f>IF(B54="SI", "REGULAR", "PENDIENTE")</f>
+        <v/>
+      </c>
+      <c r="F54" s="10">
+        <f>IF(C54="SI", "APROBADO", IF(B54="SI", "ADEUDA FINAL", "ADEUDA"))</f>
+        <v/>
+      </c>
+      <c r="G54" s="11">
+        <f>IF(C54="SI", "🟢 Aprobada", IF(B54="SI", "🟡 Regular", "🟣 Pendiente"))</f>
         <v/>
       </c>
     </row>
@@ -2295,22 +2260,22 @@
     <mergeCell ref="I12:J12"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A27:G27"/>
-    <mergeCell ref="I3:J3"/>
     <mergeCell ref="I15:J15"/>
-    <mergeCell ref="I16:J16"/>
+    <mergeCell ref="I10:J10"/>
     <mergeCell ref="A46:G46"/>
-    <mergeCell ref="A4:G4"/>
     <mergeCell ref="A50:G50"/>
+    <mergeCell ref="I1:K1"/>
     <mergeCell ref="I11:J11"/>
+    <mergeCell ref="A16:G16"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A15:G15"/>
     <mergeCell ref="I13:J13"/>
     <mergeCell ref="I14:J14"/>
-    <mergeCell ref="I17:J17"/>
+    <mergeCell ref="I9:J9"/>
+    <mergeCell ref="A5:G5"/>
     <mergeCell ref="A37:G37"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="B4:C54" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B6 B7 B8 B9 B10 B11 B12 B13 B14 B15 B17 B18 B19 B20 B21 B22 B23 B24 B25 B26 B28 B29 B30 B31 B32 B33 B34 B35 B36 B38 B39 B40 B41 B42 B43 B44 B45 B47 B48 B49 B51 B52 B53 B54 C6 C7 C8 C9 C10 C11 C12 C13 C14 C15 C17 C18 C19 C20 C21 C22 C23 C24 C25 C26 C28 C29 C30 C31 C32 C33 C34 C35 C36 C38 C39 C40 C41 C42 C43 C44 C45 C47 C48 C49 C51 C52 C53 C54" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Opción inválida" error="Por favor, elegí 'SI' o 'NO' de la lista desplegable." type="list">
       <formula1>"SI,NO"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>